<commit_message>
reconciled projects tracker, generated 22 project database JSON files, updated app logo, and fixed TS sidebar type compile errors
</commit_message>
<xml_diff>
--- a/Projects_2026.xlsx
+++ b/Projects_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAM\Documents\Antigravity\Englabs Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D700E32-2380-41E4-AF59-E0CE1FE568A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D4B74A-953B-43D6-8EEB-CBB0B08A363B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects 2026" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Projects 2026'!$A$1:$A$28</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="100">
   <si>
     <t>ENGLABS PROJECTS 2026</t>
   </si>
@@ -116,9 +116,6 @@
   </si>
   <si>
     <t>C5283</t>
-  </si>
-  <si>
-    <t>00/09</t>
   </si>
   <si>
     <t>C5286</t>
@@ -447,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -481,6 +478,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,11 +795,11 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12" style="13" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="8" max="8" width="14" style="13" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
     <col min="12" max="12" width="16" customWidth="1"/>
@@ -834,7 +840,7 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="13" t="s">
         <v>5</v>
       </c>
       <c r="E3" t="s">
@@ -846,7 +852,7 @@
       <c r="G3" t="s">
         <v>8</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="13" t="s">
         <v>9</v>
       </c>
       <c r="I3" t="s">
@@ -920,20 +926,20 @@
       <c r="C5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="14">
         <v>5</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="G5" s="5">
         <v>0</v>
       </c>
-      <c r="H5" s="5">
-        <v>5</v>
+      <c r="H5" s="14">
+        <v>2</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4" t="s">
@@ -962,20 +968,20 @@
       <c r="C6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="15">
         <v>9</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G6" s="9">
         <v>0</v>
       </c>
-      <c r="H6" s="9">
-        <v>9</v>
+      <c r="H6" s="15">
+        <v>5</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8" t="s">
@@ -996,15 +1002,15 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="5">
+      <c r="D7" s="14">
         <v>10</v>
       </c>
       <c r="E7" s="3"/>
@@ -1014,7 +1020,7 @@
       <c r="G7" s="5">
         <v>0</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="14">
         <v>10</v>
       </c>
       <c r="I7" s="4" t="s">
@@ -1038,38 +1044,38 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="9">
+      <c r="D8" s="15">
         <v>15</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0</v>
+      </c>
+      <c r="H8" s="15">
+        <v>15</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="G8" s="9">
-        <v>0</v>
-      </c>
-      <c r="H8" s="9">
-        <v>15</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>38</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>21</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M8" s="8" t="s">
         <v>23</v>
@@ -1080,37 +1086,37 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="14">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="5">
+      <c r="F9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="5">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14">
         <v>14</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="5">
-        <v>14</v>
-      </c>
       <c r="I9" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J9" s="4" t="s">
         <v>21</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L9" s="4" t="s">
         <v>22</v>
@@ -1124,25 +1130,25 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="9">
+      <c r="D10" s="15">
         <v>1000</v>
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G10" s="9">
         <v>250</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="15">
         <v>750</v>
       </c>
       <c r="I10" s="8" t="s">
@@ -1152,7 +1158,7 @@
         <v>22</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L10" s="8" t="s">
         <v>22</v>
@@ -1166,40 +1172,40 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="14">
+        <v>150</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="5">
-        <v>150</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="G11" s="5">
         <v>141</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="14">
         <v>9</v>
       </c>
       <c r="I11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K11" s="4" t="s">
+      <c r="L11" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>23</v>
@@ -1210,40 +1216,40 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="D12" s="15">
+        <v>8</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="9">
+      <c r="F12" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="9">
+        <v>0</v>
+      </c>
+      <c r="H12" s="15">
         <v>8</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G12" s="9">
-        <v>0</v>
-      </c>
-      <c r="H12" s="9">
-        <v>8</v>
-      </c>
       <c r="I12" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M12" s="8" t="s">
         <v>23</v>
@@ -1254,40 +1260,40 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="14">
+        <v>11</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="5">
+      <c r="F13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="5">
+        <v>0</v>
+      </c>
+      <c r="H13" s="14">
         <v>11</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" s="5">
-        <v>0</v>
-      </c>
-      <c r="H13" s="5">
-        <v>11</v>
-      </c>
       <c r="I13" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J13" s="4" t="s">
         <v>21</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>23</v>
@@ -1298,31 +1304,31 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="8" t="s">
+      <c r="D14" s="15">
+        <v>32</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D14" s="9">
+      <c r="F14" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="9">
+        <v>0</v>
+      </c>
+      <c r="H14" s="15">
         <v>32</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G14" s="9">
-        <v>0</v>
-      </c>
-      <c r="H14" s="9">
-        <v>32</v>
-      </c>
       <c r="I14" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>21</v>
@@ -1342,27 +1348,27 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="14">
+        <v>36</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="5">
-        <v>36</v>
-      </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="G15" s="5">
         <v>0</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="14">
         <v>36</v>
       </c>
       <c r="I15" s="4" t="s">
@@ -1386,27 +1392,27 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" s="8" t="s">
+      <c r="D16" s="15">
+        <v>4</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="D16" s="9">
-        <v>4</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>74</v>
-      </c>
       <c r="G16" s="9">
         <v>0</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="15">
         <v>4</v>
       </c>
       <c r="I16" s="8" t="s">
@@ -1430,19 +1436,19 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="14">
+        <v>5</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D17" s="5">
-        <v>5</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>29</v>
@@ -1450,20 +1456,20 @@
       <c r="G17" s="5">
         <v>0</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="14">
         <v>5</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J17" s="4" t="s">
         <v>21</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M17" s="4" t="s">
         <v>23</v>
@@ -1474,19 +1480,19 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D18" s="15">
+        <v>5</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>79</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="9">
-        <v>5</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>80</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>29</v>
@@ -1494,11 +1500,11 @@
       <c r="G18" s="9">
         <v>0</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="15">
         <v>5</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J18" s="8" t="s">
         <v>21</v>
@@ -1518,31 +1524,31 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="14">
+        <v>2</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D19" s="5">
+      <c r="G19" s="5">
+        <v>0</v>
+      </c>
+      <c r="H19" s="14">
         <v>2</v>
       </c>
-      <c r="E19" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="G19" s="5">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5">
-        <v>2</v>
-      </c>
       <c r="I19" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J19" s="4" t="s">
         <v>21</v>
@@ -1562,31 +1568,31 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="C20" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="15">
+        <v>48</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20" s="9">
+      <c r="G20" s="9">
+        <v>0</v>
+      </c>
+      <c r="H20" s="15">
         <v>48</v>
       </c>
-      <c r="E20" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="G20" s="9">
-        <v>0</v>
-      </c>
-      <c r="H20" s="9">
-        <v>48</v>
-      </c>
       <c r="I20" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>21</v>
@@ -1606,27 +1612,27 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="14">
+        <v>90</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D21" s="5">
-        <v>90</v>
-      </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>90</v>
-      </c>
       <c r="G21" s="5">
         <v>0</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="14">
         <v>90</v>
       </c>
       <c r="I21" s="4" t="s">
@@ -1636,10 +1642,10 @@
         <v>21</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M21" s="4" t="s">
         <v>23</v>
@@ -1650,25 +1656,25 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" s="9">
+      <c r="D22" s="15">
         <v>55</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G22" s="9">
         <v>15</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="15">
         <v>40</v>
       </c>
       <c r="I22" s="8"/>
@@ -1688,25 +1694,25 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D23" s="5">
+        <v>93</v>
+      </c>
+      <c r="D23" s="14">
         <v>55</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G23" s="5">
         <v>40</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="14">
         <v>15</v>
       </c>
       <c r="I23" s="4"/>
@@ -1727,22 +1733,22 @@
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
       <c r="B24" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="9">
+        <v>91</v>
+      </c>
+      <c r="D24" s="15">
         <v>125</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G24" s="9">
         <v>0</v>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="15">
         <v>125</v>
       </c>
       <c r="I24" s="8"/>
@@ -1757,28 +1763,28 @@
         <v>23</v>
       </c>
       <c r="N24" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D25" s="5">
+        <v>93</v>
+      </c>
+      <c r="D25" s="14">
         <v>125</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G25" s="5">
         <v>0</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="14">
         <v>125</v>
       </c>
       <c r="I25" s="4"/>
@@ -1793,28 +1799,28 @@
         <v>23</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
       <c r="B26" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D26" s="9">
+        <v>97</v>
+      </c>
+      <c r="D26" s="15">
         <v>100</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G26" s="9">
         <v>0</v>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="15">
         <v>100</v>
       </c>
       <c r="I26" s="8"/>
@@ -1829,28 +1835,28 @@
         <v>23</v>
       </c>
       <c r="N26" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D27" s="5">
+        <v>99</v>
+      </c>
+      <c r="D27" s="14">
         <v>100</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G27" s="5">
         <v>0</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="14">
         <v>100</v>
       </c>
       <c r="I27" s="4"/>
@@ -1865,18 +1871,18 @@
         <v>23</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
+      <c r="D28" s="15"/>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
       <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
+      <c r="H28" s="15"/>
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>

</xml_diff>